<commit_message>
fix(schema): some fixes and enrichment
</commit_message>
<xml_diff>
--- a/project/excel/oscal_assessment_plan.xlsx
+++ b/project/excel/oscal_assessment_plan.xlsx
@@ -850,11 +850,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"home,office,mobile"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -901,11 +896,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="A2:A1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"home,work"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -932,11 +922,6 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SHA-224,SHA-256,SHA-384,SHA-512,SHA3-224,SHA3-256,SHA3-384,SHA3-512"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>